<commit_message>
đang kiểm thử chương trình
</commit_message>
<xml_diff>
--- a/Nền tảng vận hành trạm sạc xe điện (CSMS).xlsx
+++ b/Nền tảng vận hành trạm sạc xe điện (CSMS).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TTCS_K8S4_N5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC44C80-8235-402A-A969-1CFBC2E95376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C203EF-1EA1-41F9-B1E6-92318ADAF032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Thông tin" sheetId="1" r:id="rId1"/>
@@ -6539,6 +6539,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6605,7 +6606,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>120</v>
       </c>
@@ -6652,7 +6653,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>126</v>
       </c>
@@ -6699,7 +6700,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>132</v>
       </c>
@@ -6744,7 +6745,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>138</v>
       </c>
@@ -6791,7 +6792,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>144</v>
       </c>
@@ -6838,7 +6839,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>149</v>
       </c>
@@ -6883,7 +6884,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>154</v>
       </c>
@@ -6930,7 +6931,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>159</v>
       </c>
@@ -6977,7 +6978,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>164</v>
       </c>
@@ -7022,7 +7023,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="165" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>170</v>
       </c>
@@ -7586,7 +7587,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="210" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>232</v>
       </c>
@@ -7633,7 +7634,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="210" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>238</v>
       </c>
@@ -7680,7 +7681,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="165" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>243</v>
       </c>
@@ -7727,7 +7728,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>248</v>
       </c>
@@ -7774,7 +7775,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="255" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>130</v>
       </c>
@@ -7821,7 +7822,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="165" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>258</v>
       </c>
@@ -7868,7 +7869,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>264</v>
       </c>
@@ -7915,7 +7916,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>269</v>
       </c>
@@ -7960,7 +7961,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>274</v>
       </c>
@@ -8007,7 +8008,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>280</v>
       </c>
@@ -8054,7 +8055,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="165" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>285</v>
       </c>
@@ -8101,7 +8102,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>291</v>
       </c>
@@ -8148,7 +8149,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>296</v>
       </c>
@@ -8195,7 +8196,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>301</v>
       </c>
@@ -8242,7 +8243,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>307</v>
       </c>
@@ -8289,7 +8290,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>312</v>
       </c>
@@ -8334,7 +8335,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="195" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>319</v>
       </c>
@@ -8381,7 +8382,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>324</v>
       </c>
@@ -8428,7 +8429,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>329</v>
       </c>
@@ -8475,7 +8476,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>335</v>
       </c>
@@ -8522,7 +8523,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>341</v>
       </c>
@@ -8569,7 +8570,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>346</v>
       </c>
@@ -8616,7 +8617,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>136</v>
       </c>
@@ -8663,7 +8664,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>355</v>
       </c>
@@ -8710,7 +8711,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>361</v>
       </c>
@@ -8757,7 +8758,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>366</v>
       </c>
@@ -8804,7 +8805,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>371</v>
       </c>
@@ -8851,7 +8852,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>376</v>
       </c>
@@ -8898,7 +8899,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="51" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>381</v>
       </c>
@@ -8945,7 +8946,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>387</v>
       </c>
@@ -8992,7 +8993,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>392</v>
       </c>
@@ -9039,7 +9040,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>398</v>
       </c>
@@ -9086,7 +9087,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>403</v>
       </c>
@@ -9133,7 +9134,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>409</v>
       </c>
@@ -9180,7 +9181,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>414</v>
       </c>
@@ -9227,7 +9228,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>419</v>
       </c>
@@ -9272,7 +9273,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>424</v>
       </c>
@@ -9319,7 +9320,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>429</v>
       </c>
@@ -9366,7 +9367,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>435</v>
       </c>
@@ -9413,7 +9414,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>441</v>
       </c>
@@ -9460,7 +9461,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="63" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>446</v>
       </c>
@@ -9505,7 +9506,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>451</v>
       </c>
@@ -9552,7 +9553,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="65" spans="1:15" ht="180" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>456</v>
       </c>
@@ -9599,7 +9600,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="66" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>168</v>
       </c>
@@ -9646,7 +9647,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="67" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>467</v>
       </c>
@@ -9691,7 +9692,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="68" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>472</v>
       </c>
@@ -10669,7 +10670,13 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:O68" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:O68" xr:uid="{00000000-0009-0000-0000-000003000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="2"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>